<commit_message>
Correct Longxing outbound totals for bound bikes
</commit_message>
<xml_diff>
--- a/dist/files/長興四站_2026年5月與9月調度量比較.xlsx
+++ b/dist/files/長興四站_2026年5月與9月調度量比較.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="調度量比較" sheetId="1" r:id="Ra09306e6649848ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日明細" sheetId="2" r:id="R8a4bc8e3311e45d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="計算說明" sheetId="3" r:id="Rb3f0a10e1fd248c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="調度量比較" sheetId="1" r:id="R322f1640f4b34d08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐日明細" sheetId="2" r:id="R468661108e0f489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="計算說明" sheetId="3" r:id="Rb4aab9000e74454a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -243,13 +243,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LongxingDailyTable" displayName="LongxingDailyTable" ref="A1:E38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LongxingDailyTable" displayName="LongxingDailyTable" ref="A1:G38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="月份"/>
     <x:tableColumn id="2" name="日期"/>
     <x:tableColumn id="3" name="6–24調入量"/>
     <x:tableColumn id="4" name="9–12調入量"/>
-    <x:tableColumn id="5" name="20–00調出量"/>
+    <x:tableColumn id="5" name="20–00毛調出量"/>
+    <x:tableColumn id="6" name="20–00配對解綁車量"/>
+    <x:tableColumn id="7" name="20–00淨調出量"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -491,11 +493,11 @@
         <x:v>6–24調入量</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!C$2:C$38)</x:f>
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!$C$2:$C$38)</x:f>
         <x:v>621</x:v>
       </x:c>
       <x:c r="C5" s="22" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!C$2:C$38)</x:f>
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!$C$2:$C$38)</x:f>
         <x:v>1028</x:v>
       </x:c>
       <x:c r="D5" s="24" t="n">
@@ -508,11 +510,11 @@
         <x:v>9–12調入量</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!D$2:D$38)</x:f>
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!$D$2:$D$38)</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="C6" s="22" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!D$2:D$38)</x:f>
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!$D$2:$D$38)</x:f>
         <x:v>453</x:v>
       </x:c>
       <x:c r="D6" s="24" t="n">
@@ -521,75 +523,137 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="19" t="str">
-        <x:v>20–00調出量</x:v>
-      </x:c>
-      <x:c r="B7" s="23" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!E$2:E$38)</x:f>
+      <x:c r="A7" s="16" t="str">
+        <x:v>20–00毛調出量</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!$E$2:$E$38)</x:f>
         <x:v>645</x:v>
       </x:c>
-      <x:c r="C7" s="23" t="n">
-        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!E$2:E$38)</x:f>
+      <x:c r="C7" s="22" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!$E$2:$E$38)</x:f>
         <x:v>627</x:v>
       </x:c>
-      <x:c r="D7" s="25" t="n">
+      <x:c r="D7" s="24" t="n">
         <x:f>C7/B7-1</x:f>
         <x:v>-0.027906976744186074</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="28" t="str">
+    <x:row r="8" ht="27" customHeight="1">
+      <x:c r="A8" s="16" t="str">
+        <x:v>20–00配對解綁車量</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!$F$2:$F$38)</x:f>
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!$F$2:$F$38)</x:f>
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D8" s="24" t="n">
+        <x:f>C8/B8-1</x:f>
+        <x:v>-0.48863636363636365</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="27" customHeight="1">
+      <x:c r="A9" s="19" t="str">
+        <x:v>20–00淨調出量（扣綁車）</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-05",'逐日明細'!$G$2:$G$38)</x:f>
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="n">
+        <x:f>SUMIF('逐日明細'!$A$2:$A$38,"2026-09",'逐日明細'!$G$2:$G$38)</x:f>
+        <x:v>582</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="n">
+        <x:f>C9/B9-1</x:f>
+        <x:v>0.044883303411131115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="28" t="str">
         <x:v>四站合計日均</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="str">
+      <x:c r="B12" s="28" t="str">
         <x:v>5月</x:v>
       </x:c>
-      <x:c r="C10" s="28" t="str">
+      <x:c r="C12" s="28" t="str">
         <x:v>9月</x:v>
       </x:c>
-      <x:c r="D10" s="28" t="str">
+      <x:c r="D12" s="28" t="str">
         <x:v>樣本日</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>6–24調入量</x:v>
-      </x:c>
-      <x:c r="B11" s="29" t="n">
-        <x:v>34.5</x:v>
-      </x:c>
-      <x:c r="C11" s="29" t="n">
-        <x:v>54.10526315789474</x:v>
-      </x:c>
-      <x:c r="D11" t="str">
-        <x:v>18／19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>9–12調入量</x:v>
-      </x:c>
-      <x:c r="B12" s="29" t="n">
-        <x:v>10.222222222222221</x:v>
-      </x:c>
-      <x:c r="C12" s="29" t="n">
-        <x:v>23.842105263157894</x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>18／19</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>20–00調出量</x:v>
+        <x:v>6–24調入量</x:v>
       </x:c>
       <x:c r="B13" s="29" t="n">
+        <x:v>34.5</x:v>
+      </x:c>
+      <x:c r="C13" s="29" t="n">
+        <x:v>54.10526315789474</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>18／19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>9–12調入量</x:v>
+      </x:c>
+      <x:c r="B14" s="29" t="n">
+        <x:v>10.222222222222221</x:v>
+      </x:c>
+      <x:c r="C14" s="29" t="n">
+        <x:v>23.842105263157894</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>18／19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>20–00毛調出量</x:v>
+      </x:c>
+      <x:c r="B15" s="29" t="n">
         <x:v>35.833333333333336</x:v>
       </x:c>
-      <x:c r="C13" s="29" t="n">
+      <x:c r="C15" s="29" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D15" t="str">
+        <x:v>18／19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>20–00配對解綁車量</x:v>
+      </x:c>
+      <x:c r="B16" s="29" t="n">
+        <x:v>4.888888888888889</x:v>
+      </x:c>
+      <x:c r="C16" s="29" t="n">
+        <x:v>2.3684210526315788</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>18／19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>20–00淨調出量（扣綁車）</x:v>
+      </x:c>
+      <x:c r="B17" s="29" t="n">
+        <x:v>30.944444444444443</x:v>
+      </x:c>
+      <x:c r="C17" s="29" t="n">
+        <x:v>30.63157894736842</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
         <x:v>18／19</x:v>
       </x:c>
     </x:row>
@@ -608,9 +672,11 @@
   <x:cols>
     <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -627,7 +693,13 @@
         <x:v>9–12調入量</x:v>
       </x:c>
       <x:c r="E1" s="9" t="str">
-        <x:v>20–00調出量</x:v>
+        <x:v>20–00毛調出量</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>20–00配對解綁車量</x:v>
+      </x:c>
+      <x:c r="G1" s="9" t="str">
+        <x:v>20–00淨調出量</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -646,6 +718,12 @@
       <x:c r="E2" t="n">
         <x:v>32</x:v>
       </x:c>
+      <x:c r="F2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G2" t="n">
+        <x:v>32</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -663,6 +741,12 @@
       <x:c r="E3" t="n">
         <x:v>14</x:v>
       </x:c>
+      <x:c r="F3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G3" t="n">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
@@ -680,6 +764,12 @@
       <x:c r="E4" t="n">
         <x:v>45</x:v>
       </x:c>
+      <x:c r="F4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" t="n">
+        <x:v>45</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -697,6 +787,12 @@
       <x:c r="E5" t="n">
         <x:v>45</x:v>
       </x:c>
+      <x:c r="F5" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="G5" t="n">
+        <x:v>31</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
@@ -714,6 +810,12 @@
       <x:c r="E6" t="n">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="F6" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G6" t="n">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
@@ -731,6 +833,12 @@
       <x:c r="E7" t="n">
         <x:v>64</x:v>
       </x:c>
+      <x:c r="F7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G7" t="n">
+        <x:v>56</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
@@ -748,6 +856,12 @@
       <x:c r="E8" t="n">
         <x:v>51</x:v>
       </x:c>
+      <x:c r="F8" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G8" t="n">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
@@ -765,6 +879,12 @@
       <x:c r="E9" t="n">
         <x:v>16</x:v>
       </x:c>
+      <x:c r="F9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" t="n">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
@@ -782,6 +902,12 @@
       <x:c r="E10" t="n">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="F10" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" t="n">
+        <x:v>48</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
@@ -799,6 +925,12 @@
       <x:c r="E11" t="n">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="F11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" t="n">
+        <x:v>48</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
@@ -816,6 +948,12 @@
       <x:c r="E12" t="n">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="F12" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" t="n">
+        <x:v>30</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
@@ -833,6 +971,12 @@
       <x:c r="E13" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
@@ -850,6 +994,12 @@
       <x:c r="E14" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G14" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -867,6 +1017,12 @@
       <x:c r="E15" t="n">
         <x:v>60</x:v>
       </x:c>
+      <x:c r="F15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" t="n">
+        <x:v>60</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -884,6 +1040,12 @@
       <x:c r="E16" t="n">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="F16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" t="n">
+        <x:v>30</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
@@ -901,6 +1063,12 @@
       <x:c r="E17" t="n">
         <x:v>34</x:v>
       </x:c>
+      <x:c r="F17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" t="n">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
@@ -918,6 +1086,12 @@
       <x:c r="E18" t="n">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="F18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" t="n">
+        <x:v>48</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
@@ -935,6 +1109,12 @@
       <x:c r="E19" t="n">
         <x:v>32</x:v>
       </x:c>
+      <x:c r="F19" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" t="n">
+        <x:v>32</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
@@ -952,6 +1132,12 @@
       <x:c r="E20" t="n">
         <x:v>61</x:v>
       </x:c>
+      <x:c r="F20" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="G20" t="n">
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
@@ -969,6 +1155,12 @@
       <x:c r="E21" t="n">
         <x:v>45</x:v>
       </x:c>
+      <x:c r="F21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" t="n">
+        <x:v>45</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
@@ -986,6 +1178,12 @@
       <x:c r="E22" t="n">
         <x:v>45</x:v>
       </x:c>
+      <x:c r="F22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>45</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
@@ -1003,6 +1201,12 @@
       <x:c r="E23" t="n">
         <x:v>48</x:v>
       </x:c>
+      <x:c r="F23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" t="n">
+        <x:v>48</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -1020,6 +1224,12 @@
       <x:c r="E24" t="n">
         <x:v>34</x:v>
       </x:c>
+      <x:c r="F24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" t="n">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
@@ -1037,6 +1247,12 @@
       <x:c r="E25" t="n">
         <x:v>12</x:v>
       </x:c>
+      <x:c r="F25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G25" t="n">
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
@@ -1054,6 +1270,12 @@
       <x:c r="E26" t="n">
         <x:v>50</x:v>
       </x:c>
+      <x:c r="F26" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" t="n">
+        <x:v>50</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
@@ -1071,6 +1293,12 @@
       <x:c r="E27" t="n">
         <x:v>66</x:v>
       </x:c>
+      <x:c r="F27" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" t="n">
+        <x:v>66</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
@@ -1088,6 +1316,12 @@
       <x:c r="E28" t="n">
         <x:v>34</x:v>
       </x:c>
+      <x:c r="F28" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" t="n">
+        <x:v>34</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
@@ -1105,6 +1339,12 @@
       <x:c r="E29" t="n">
         <x:v>46</x:v>
       </x:c>
+      <x:c r="F29" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" t="n">
+        <x:v>46</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
@@ -1122,6 +1362,12 @@
       <x:c r="E30" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F30" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
@@ -1139,6 +1385,12 @@
       <x:c r="E31" t="n">
         <x:v>44</x:v>
       </x:c>
+      <x:c r="F31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>44</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
@@ -1156,6 +1408,12 @@
       <x:c r="E32" t="n">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="F32" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" t="n">
+        <x:v>30</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
@@ -1173,6 +1431,12 @@
       <x:c r="E33" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F33" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
@@ -1190,6 +1454,12 @@
       <x:c r="E34" t="n">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="F34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
@@ -1207,6 +1477,12 @@
       <x:c r="E35" t="n">
         <x:v>17</x:v>
       </x:c>
+      <x:c r="F35" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" t="n">
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
@@ -1224,6 +1500,12 @@
       <x:c r="E36" t="n">
         <x:v>50</x:v>
       </x:c>
+      <x:c r="F36" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G36" t="n">
+        <x:v>50</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
@@ -1241,6 +1523,12 @@
       <x:c r="E37" t="n">
         <x:v>28</x:v>
       </x:c>
+      <x:c r="F37" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G37" t="n">
+        <x:v>28</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
@@ -1256,13 +1544,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E38" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F38" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G38" t="n">
         <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82447077937e40d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree3ced40b0a4455d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1351,46 +1645,68 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="32" t="str">
-        <x:v>20–00調出</x:v>
+        <x:v>20–00毛調出</x:v>
       </x:c>
       <x:c r="B9" s="32" t="str">
         <x:v>20:00–23:59</x:v>
       </x:c>
       <x:c r="C9" s="32" t="str">
-        <x:v>四站調出數量合計後除以樣本日</x:v>
+        <x:v>工作狀態=調出的四站數量合計</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="32" t="str">
-        <x:v>VDS篩選</x:v>
+        <x:v>配對解綁車</x:v>
       </x:c>
       <x:c r="B10" s="32" t="str">
-        <x:v>工作狀態=調入／調出；車種=2.0／2.0E；數量&gt;0</x:v>
+        <x:v>同站＋同車號＋同車種＋同抵達秒數</x:v>
       </x:c>
       <x:c r="C10" s="32" t="str">
-        <x:v>依車號＋站碼＋狀態＋車種＋數量＋抵達時間去重</x:v>
+        <x:v>每組扣除 min(調出, 解綁車)；9筆全部配對，沒有未匹配</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32" t="str">
-        <x:v>5月總量</x:v>
+        <x:v>20–00淨調出</x:v>
       </x:c>
       <x:c r="B11" s="32" t="str">
-        <x:v>621／184／645</x:v>
+        <x:v>毛調出－配對解綁車</x:v>
       </x:c>
       <x:c r="C11" s="32" t="str">
-        <x:v>依序為6–24調入、9–12調入、20–00調出</x:v>
+        <x:v>排除原綁車先解綁再調出的車輛</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32" t="str">
+        <x:v>VDS篩選</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>車種=2.0／2.0E；數量&gt;0</x:v>
+      </x:c>
+      <x:c r="C12" s="32" t="str">
+        <x:v>原始列依車號＋站碼＋狀態＋車種＋數量＋抵達時間去重</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="32" t="str">
+        <x:v>5月總量</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>621／184／645／88／557</x:v>
+      </x:c>
+      <x:c r="C13" s="32" t="str">
+        <x:v>依序為6–24調入、9–12調入、毛調出、配對解綁、淨調出</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="32" t="str">
         <x:v>9月總量</x:v>
       </x:c>
-      <x:c r="B12" s="32" t="str">
-        <x:v>1,028／453／627</x:v>
-      </x:c>
-      <x:c r="C12" s="32" t="str">
-        <x:v>依序為6–24調入、9–12調入、20–00調出</x:v>
+      <x:c r="B14" s="32" t="str">
+        <x:v>1,028／453／627／45／582</x:v>
+      </x:c>
+      <x:c r="C14" s="32" t="str">
+        <x:v>依序為6–24調入、9–12調入、毛調出、配對解綁、淨調出</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>